<commit_message>
Sample deal: schools, FMV and trade-out read internal-only (restage re-run)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/downloads/underwriting-demo/sample-deal-summary.xlsx
+++ b/public/downloads/underwriting-demo/sample-deal-summary.xlsx
@@ -1079,7 +1079,7 @@
       </c>
       <c r="D42" s="6" t="inlineStr">
         <is>
-          <t>Not stated in the uploaded documents</t>
+          <t>Internal pipeline only</t>
         </is>
       </c>
     </row>
@@ -1387,7 +1387,7 @@
       </c>
       <c r="D65" s="6" t="inlineStr">
         <is>
-          <t>Not stated in the uploaded documents</t>
+          <t>Internal pipeline only</t>
         </is>
       </c>
     </row>
@@ -1426,7 +1426,7 @@
       </c>
       <c r="D67" s="6" t="inlineStr">
         <is>
-          <t>Not stated in the uploaded documents</t>
+          <t>Internal pipeline only</t>
         </is>
       </c>
     </row>
@@ -1465,7 +1465,7 @@
       </c>
       <c r="D69" s="6" t="inlineStr">
         <is>
-          <t>Not stated in the uploaded documents</t>
+          <t>Internal pipeline only</t>
         </is>
       </c>
     </row>
@@ -18194,7 +18194,7 @@
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Not stated in the uploaded documents</t>
+          <t>Internal pipeline only</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
@@ -18210,7 +18210,7 @@
       <c r="F28" s="12" t="n"/>
       <c r="G28" s="22" t="inlineStr">
         <is>
-          <t>No uploaded document stated this, so the value reads MISSING. Nothing was assumed to fill it.</t>
+          <t>The internal pipeline pulls a market value by web lookup; the demo does not reach the web.</t>
         </is>
       </c>
     </row>
@@ -18468,7 +18468,7 @@
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>Not stated in the uploaded documents</t>
+          <t>Internal pipeline only</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
@@ -18484,7 +18484,7 @@
       <c r="F36" s="12" t="n"/>
       <c r="G36" s="22" t="inlineStr">
         <is>
-          <t>No uploaded document stated this, so the value reads MISSING. Nothing was assumed to fill it.</t>
+          <t>The internal pipeline looks up the attendance-zone elementary, middle and high school and their public ratings; the demo reads a school name only where the memorandum states one and never rates it.</t>
         </is>
       </c>
     </row>
@@ -18501,7 +18501,7 @@
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Not stated in the uploaded documents</t>
+          <t>Internal pipeline only</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
@@ -18517,7 +18517,7 @@
       <c r="F37" s="12" t="n"/>
       <c r="G37" s="22" t="inlineStr">
         <is>
-          <t>No uploaded document stated this, so the value reads MISSING. Nothing was assumed to fill it.</t>
+          <t>The internal pipeline looks up the attendance-zone elementary, middle and high school and their public ratings; the demo reads a school name only where the memorandum states one and never rates it.</t>
         </is>
       </c>
     </row>
@@ -18534,7 +18534,7 @@
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>Not stated in the uploaded documents</t>
+          <t>Internal pipeline only</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
@@ -18550,7 +18550,7 @@
       <c r="F38" s="12" t="n"/>
       <c r="G38" s="22" t="inlineStr">
         <is>
-          <t>No uploaded document stated this, so the value reads MISSING. Nothing was assumed to fill it.</t>
+          <t>The internal pipeline looks up the attendance-zone elementary, middle and high school and their public ratings; the demo reads a school name only where the memorandum states one and never rates it.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sample tabs regrouped per Herman: rent comps, property tax and supply as their own sections; raw / analysis / audit trail per statement; Excel model group; no notes tab
Deal name is the real one with illustrative party names; summary card drops deal status,
notes and excluded-by-design; internal-only values read 'Available in the internal
underwriting agent only'; manifest is Name / Value / Source / Fills in the model; pricing
moved to the T-12 analysis tab; new rent-roll audit-trail fragment.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/downloads/underwriting-demo/sample-deal-summary.xlsx
+++ b/public/downloads/underwriting-demo/sample-deal-summary.xlsx
@@ -537,7 +537,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Southern Avenue Sample — as of 2026-08-31</t>
+          <t>505 West — as of 2026-08-31</t>
         </is>
       </c>
     </row>
@@ -575,12 +575,12 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Southern Avenue Sample</t>
+          <t>505 West</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>Illustrative</t>
+          <t>Sample Property Offering Memorandum.pdf — p.3</t>
         </is>
       </c>
     </row>
@@ -854,12 +854,12 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Institutional owner-operator (name withheld)</t>
+          <t>Sonoran Residential Holdings LLC</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>Sample Property Offering Memorandum.pdf — withheld</t>
+          <t>Illustrative name</t>
         </is>
       </c>
     </row>
@@ -871,12 +871,12 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Listing brokerage</t>
+          <t>Desert Ridge Capital Advisors</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>Sample Property Offering Memorandum.pdf — withheld</t>
+          <t>Illustrative name</t>
         </is>
       </c>
     </row>
@@ -1503,7 +1503,7 @@
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>This sample is a real, previously marketed multifamily asset's statements, perturbed: trailing-twelve income lines are 10% higher and expense lines 5% lower than the originals, rent-roll rents are 5% higher and lease dates one month earlier, and the pricing is illustrative. The property facts — unit mix, vintage, size — are the real ones. The ADDRESS is illustrative: 2151 E Southern Ave, Mesa, AZ 85204 is not the asset's location, and the demand, supply, rent-comp and property-tax tabs were pulled for this illustrative address from the same sources a live upload reads. The asset's name, its seller and its brokerage are withheld.</t>
+          <t>This sample is a real, previously marketed multifamily asset's statements, perturbed: trailing-twelve income lines are 10% higher and expense lines 5% lower than the originals, rent-roll rents are 5% higher and lease dates one month earlier, and the pricing is illustrative. The property facts — unit mix, vintage, size — are the real ones. The ADDRESS is illustrative: 2151 E Southern Ave, Mesa, AZ 85204 is not the asset's location, and the demand, supply, rent-comp and property-tax tabs were pulled for this illustrative address from the same sources a live upload reads. The seller and brokerage names are illustrative; the real parties are withheld.</t>
         </is>
       </c>
     </row>
@@ -1592,7 +1592,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Southern Avenue Sample — as of 2026-09-03</t>
+          <t>505 West — as of 2026-09-03</t>
         </is>
       </c>
     </row>
@@ -13648,7 +13648,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Southern Avenue Sample — as of 2026-08-31</t>
+          <t>505 West — as of 2026-08-31</t>
         </is>
       </c>
     </row>
@@ -14141,7 +14141,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Southern Avenue Sample — as of 2026-08-31</t>
+          <t>505 West — as of 2026-08-31</t>
         </is>
       </c>
     </row>
@@ -16408,7 +16408,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Southern Avenue Sample — as of 2026-08-31</t>
+          <t>505 West — as of 2026-08-31</t>
         </is>
       </c>
     </row>
@@ -16745,7 +16745,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Southern Avenue Sample — as of 2026-08-31</t>
+          <t>505 West — as of 2026-08-31</t>
         </is>
       </c>
     </row>
@@ -17000,7 +17000,7 @@
       </c>
       <c r="C18" s="22" t="inlineStr">
         <is>
-          <t>This sample is a real, previously marketed multifamily asset's statements, perturbed: trailing-twelve income lines are 10% higher and expense lines 5% lower than the originals, rent-roll rents are 5% higher and lease dates one month earlier, and the pricing is illustrative. The property facts — unit mix, vintage, size — are the real ones. The ADDRESS is illustrative: 2151 E Southern Ave, Mesa, AZ 85204 is not the asset's location, and the demand, supply, rent-comp and property-tax tabs were pulled for this illustrative address from the same sources a live upload reads. The asset's name, its seller and its brokerage are withheld.</t>
+          <t>This sample is a real, previously marketed multifamily asset's statements, perturbed: trailing-twelve income lines are 10% higher and expense lines 5% lower than the originals, rent-roll rents are 5% higher and lease dates one month earlier, and the pricing is illustrative. The property facts — unit mix, vintage, size — are the real ones. The ADDRESS is illustrative: 2151 E Southern Ave, Mesa, AZ 85204 is not the asset's location, and the demand, supply, rent-comp and property-tax tabs were pulled for this illustrative address from the same sources a live upload reads. The seller and brokerage names are illustrative; the real parties are withheld.</t>
         </is>
       </c>
     </row>
@@ -17462,7 +17462,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Southern Avenue Sample — as of 2026-08-31</t>
+          <t>505 West — as of 2026-08-31</t>
         </is>
       </c>
     </row>
@@ -18090,17 +18090,17 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Southern Avenue Sample</t>
+          <t>505 West</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Illustrative</t>
+          <t>Sample Property Offering Memorandum.pdf</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>p.3</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
@@ -18111,7 +18111,7 @@
       <c r="F25" s="12" t="n"/>
       <c r="G25" s="22" t="inlineStr">
         <is>
-          <t>The sample's name is illustrative; the asset's real name is withheld.</t>
+          <t>The deal name as the memorandum states it.</t>
         </is>
       </c>
     </row>
@@ -18259,17 +18259,17 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Listing brokerage</t>
+          <t>Desert Ridge Capital Advisors</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>Sample Property Offering Memorandum.pdf</t>
+          <t>Illustrative name</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>withheld</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
@@ -18280,7 +18280,7 @@
       <c r="F30" s="12" t="n"/>
       <c r="G30" s="22" t="inlineStr">
         <is>
-          <t>Stated in the memorandum; withheld from the public sample because it identifies the real asset.</t>
+          <t>An illustrative name. The real party is withheld from the public sample.</t>
         </is>
       </c>
     </row>
@@ -18562,17 +18562,17 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>Institutional owner-operator (name withheld)</t>
+          <t>Sonoran Residential Holdings LLC</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Sample Property Offering Memorandum.pdf</t>
+          <t>Illustrative name</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>withheld</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
@@ -18583,7 +18583,7 @@
       <c r="F39" s="12" t="n"/>
       <c r="G39" s="22" t="inlineStr">
         <is>
-          <t>Stated in the memorandum; withheld from the public sample because it identifies the real asset.</t>
+          <t>An illustrative name. The real party is withheld from the public sample.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sample card fixes: no status / price-per-unit / FMV, year-one tax, schools with ratings; fine print and perturbation wording removed
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/downloads/underwriting-demo/sample-deal-summary.xlsx
+++ b/public/downloads/underwriting-demo/sample-deal-summary.xlsx
@@ -1377,17 +1377,12 @@
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>Internal pipeline only</t>
-        </is>
-      </c>
-      <c r="C65" s="6" t="inlineStr">
-        <is>
-          <t>The internal pipeline looks up the attendance-zone elementary, middle and high school and their public ratings; the demo reads a school name only where the memorandum states one and never rates it.</t>
+          <t>Porter Elementary School</t>
         </is>
       </c>
       <c r="D65" s="6" t="inlineStr">
         <is>
-          <t>Internal pipeline only</t>
+          <t>Internal underwriting agent — attendance-zone school lookup — 2151 E Southern Ave, Mesa, AZ 85204 on 2026-09-14</t>
         </is>
       </c>
     </row>
@@ -1397,15 +1392,8 @@
           <t>Elementary rating</t>
         </is>
       </c>
-      <c r="B66" s="5" t="inlineStr">
-        <is>
-          <t>Internal pipeline only</t>
-        </is>
-      </c>
-      <c r="C66" s="6" t="inlineStr">
-        <is>
-          <t>The internal pipeline looks up the attendance-zone elementary, middle and high school and their public ratings; the demo reads a school name only where the memorandum states one and never rates it.</t>
-        </is>
+      <c r="B66" s="8" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="67">
@@ -1416,17 +1404,12 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>Internal pipeline only</t>
-        </is>
-      </c>
-      <c r="C67" s="6" t="inlineStr">
-        <is>
-          <t>The internal pipeline looks up the attendance-zone elementary, middle and high school and their public ratings; the demo reads a school name only where the memorandum states one and never rates it.</t>
+          <t>Taylor Junior High School</t>
         </is>
       </c>
       <c r="D67" s="6" t="inlineStr">
         <is>
-          <t>Internal pipeline only</t>
+          <t>Internal underwriting agent — attendance-zone school lookup — 2151 E Southern Ave, Mesa, AZ 85204 on 2026-09-14</t>
         </is>
       </c>
     </row>
@@ -1436,15 +1419,8 @@
           <t>Middle rating</t>
         </is>
       </c>
-      <c r="B68" s="5" t="inlineStr">
-        <is>
-          <t>Internal pipeline only</t>
-        </is>
-      </c>
-      <c r="C68" s="6" t="inlineStr">
-        <is>
-          <t>The internal pipeline looks up the attendance-zone elementary, middle and high school and their public ratings; the demo reads a school name only where the memorandum states one and never rates it.</t>
-        </is>
+      <c r="B68" s="8" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="69">
@@ -1455,17 +1431,12 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>Internal pipeline only</t>
-        </is>
-      </c>
-      <c r="C69" s="6" t="inlineStr">
-        <is>
-          <t>The internal pipeline looks up the attendance-zone elementary, middle and high school and their public ratings; the demo reads a school name only where the memorandum states one and never rates it.</t>
+          <t>Mesa High School</t>
         </is>
       </c>
       <c r="D69" s="6" t="inlineStr">
         <is>
-          <t>Internal pipeline only</t>
+          <t>Internal underwriting agent — attendance-zone school lookup — 2151 E Southern Ave, Mesa, AZ 85204 on 2026-09-14</t>
         </is>
       </c>
     </row>
@@ -1475,15 +1446,8 @@
           <t>High rating</t>
         </is>
       </c>
-      <c r="B70" s="5" t="inlineStr">
-        <is>
-          <t>Internal pipeline only</t>
-        </is>
-      </c>
-      <c r="C70" s="6" t="inlineStr">
-        <is>
-          <t>The internal pipeline looks up the attendance-zone elementary, middle and high school and their public ratings; the demo reads a school name only where the memorandum states one and never rates it.</t>
-        </is>
+      <c r="B70" s="8" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="72">
@@ -1503,7 +1467,7 @@
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>This sample is a real, previously marketed multifamily asset's statements, perturbed: trailing-twelve income lines are 10% higher and expense lines 5% lower than the originals, rent-roll rents are 5% higher and lease dates one month earlier, and the pricing is illustrative. The property facts — unit mix, vintage, size — are the real ones. The ADDRESS is illustrative: 2151 E Southern Ave, Mesa, AZ 85204 is not the asset's location, and the demand, supply, rent-comp and property-tax tabs were pulled for this illustrative address from the same sources a live upload reads. The seller and brokerage names are illustrative; the real parties are withheld.</t>
+          <t>The address shown is illustrative and is not the asset's location; the demand, supply, rent-comp and property-tax tabs were pulled for this illustrative address from the same sources a live upload reads. The seller and brokerage names are illustrative; the real parties are withheld. Pricing is illustrative.</t>
         </is>
       </c>
     </row>
@@ -16990,7 +16954,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>This sample is a real deal, perturbed, at an illustrative address</t>
+          <t>This sample sits at an illustrative address</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
@@ -17000,7 +16964,7 @@
       </c>
       <c r="C18" s="22" t="inlineStr">
         <is>
-          <t>This sample is a real, previously marketed multifamily asset's statements, perturbed: trailing-twelve income lines are 10% higher and expense lines 5% lower than the originals, rent-roll rents are 5% higher and lease dates one month earlier, and the pricing is illustrative. The property facts — unit mix, vintage, size — are the real ones. The ADDRESS is illustrative: 2151 E Southern Ave, Mesa, AZ 85204 is not the asset's location, and the demand, supply, rent-comp and property-tax tabs were pulled for this illustrative address from the same sources a live upload reads. The seller and brokerage names are illustrative; the real parties are withheld.</t>
+          <t>The address shown is illustrative and is not the asset's location; the demand, supply, rent-comp and property-tax tabs were pulled for this illustrative address from the same sources a live upload reads. The seller and brokerage names are illustrative; the real parties are withheld. Pricing is illustrative.</t>
         </is>
       </c>
     </row>
@@ -18463,17 +18427,17 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>Porter Elementary School</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>Internal pipeline only</t>
+          <t>Internal underwriting agent — attendance-zone school lookup</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2151 E Southern Ave, Mesa, AZ 85204 on 2026-09-14</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -18484,7 +18448,7 @@
       <c r="F36" s="12" t="n"/>
       <c r="G36" s="22" t="inlineStr">
         <is>
-          <t>The internal pipeline looks up the attendance-zone elementary, middle and high school and their public ratings; the demo reads a school name only where the memorandum states one and never rates it.</t>
+          <t>Looked up for the illustrative address by the internal underwriting agent; the public demo does not run this on an uploaded deal.</t>
         </is>
       </c>
     </row>
@@ -18496,17 +18460,17 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>Mesa High School</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Internal pipeline only</t>
+          <t>Internal underwriting agent — attendance-zone school lookup</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2151 E Southern Ave, Mesa, AZ 85204 on 2026-09-14</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
@@ -18517,7 +18481,7 @@
       <c r="F37" s="12" t="n"/>
       <c r="G37" s="22" t="inlineStr">
         <is>
-          <t>The internal pipeline looks up the attendance-zone elementary, middle and high school and their public ratings; the demo reads a school name only where the memorandum states one and never rates it.</t>
+          <t>Looked up for the illustrative address by the internal underwriting agent; the public demo does not run this on an uploaded deal.</t>
         </is>
       </c>
     </row>
@@ -18529,17 +18493,17 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>Taylor Junior High School</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>Internal pipeline only</t>
+          <t>Internal underwriting agent — attendance-zone school lookup</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2151 E Southern Ave, Mesa, AZ 85204 on 2026-09-14</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
@@ -18550,7 +18514,7 @@
       <c r="F38" s="12" t="n"/>
       <c r="G38" s="22" t="inlineStr">
         <is>
-          <t>The internal pipeline looks up the attendance-zone elementary, middle and high school and their public ratings; the demo reads a school name only where the memorandum states one and never rates it.</t>
+          <t>Looked up for the illustrative address by the internal underwriting agent; the public demo does not run this on an uploaded deal.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sample set re-restaged: reconciliation PASS on the rent-roll audit trail, statement sanity checks and the trailing T-3 series on the T-12 tabs, duplicate rows disclosed
The refooted sample materials (the export's totals row and per-status summary now foot to the
scaled unit rows) and one new pipeline run; nine E2 rules of PLAN_single_engine.md land on the
tabs. Same 14 fragments, same downloads, no page code change.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/downloads/underwriting-demo/sample-deal-summary.xlsx
+++ b/public/downloads/underwriting-demo/sample-deal-summary.xlsx
@@ -725,7 +725,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>garden-style multifamily</t>
+          <t>Garden-style multifamily</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
@@ -794,7 +794,7 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>One-, two-, and three-bedroom residences averaging 856 square feet across 40 buildings on 15.87 acres</t>
+          <t>Diversified mix of one-, two-, and three-bedroom residences averaging 856 square feet on approximately 15.9 acres</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
@@ -18359,7 +18359,7 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>One-, two-, and three-bedroom residences averaging 856 square feet across 40 buildings …</t>
+          <t>Diversified mix of one-, two-, and three-bedroom residences averaging 856 square feet o…</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
@@ -18394,7 +18394,7 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>garden-style multifamily</t>
+          <t>Garden-style multifamily</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Underwriting demo: sample outputs use the rent roll's signed + move-in columns
Republished via Portfolio Demo publish_to_site.py (scrub gate CLEAN) from 9b3c736 (#3300)
over 7061de9 (#3289): market rent for model = new move-in rent else in-place; the unit-mix
tab and workbook show LEASES SIGNED / NEW MOVE-IN columns instead of new-lease.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/downloads/underwriting-demo/sample-deal-summary.xlsx
+++ b/public/downloads/underwriting-demo/sample-deal-summary.xlsx
@@ -1052,7 +1052,7 @@
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>New-lease average where the plan has new leases in the lookback window, otherwise in-place. Never a blend of new and renewal.</t>
+          <t>New move-in rent (residents who moved in inside the lookback window, by move-in date) where the plan has one, otherwise in-place (in-place outright when the roll has no usable lease start or move-in date). Never a blend of new and renewal.</t>
         </is>
       </c>
       <c r="D41" s="6" t="inlineStr">
@@ -8200,7 +8200,7 @@
       </c>
       <c r="C11" s="22" t="inlineStr">
         <is>
-          <t>Market rent for the model is the new-lease average where a plan has new leases inside the lookback window, and in-place rent where it does not. It is never the average of new and renewal leases together. A blended figure reads as market rent and is not one: renewals are priced off the existing rent, so blending them in drags the number toward where rents used to be and understates the gap the underwriting is trying to measure. On an asset whose in-place rents sit above what the market is currently signing, the rule produces a market rent BELOW in-place — which is the correct and uncomfortable answer, and the one a blend would hide.</t>
+          <t>Market rent for the model is the new move-in rent — residents whose move-in date falls inside the lookback window, whatever their lease type — where a plan has one, and in-place rent where it does not. It is never the average of every lease signed, new and renewal together. A blended figure reads as market rent and is not one: renewals are priced off the existing rent, so blending them in drags the number toward where rents used to be and understates the gap the underwriting is trying to measure. On an asset whose in-place rents sit above what the market is currently signing, the rule produces a market rent BELOW in-place — which is the correct and uncomfortable answer, and the one a blend would hide.</t>
         </is>
       </c>
     </row>
@@ -8744,7 +8744,7 @@
       </c>
       <c r="C43" s="22" t="inlineStr">
         <is>
-          <t>The uploaded rent roll stated the PERIOD it covers rather than a day: as-of taken as 2026-08-31, the last day of the stated period 202608. Every window on this page (the new-lease lookback and annualised turnover) is measured back from that date, not from the day of the upload.</t>
+          <t>The uploaded rent roll stated the PERIOD it covers rather than a day: as-of taken as 2026-08-31, the last day of the stated period 202608. Every window on this page (the move-in and lease-signed lookback, and annualised turnover) is measured back from that date, not from the day of the upload.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Underwriting demo sample: community unit counts held back, years read 1984, Zillow credited on Demand
Republished via publish_to_site.py (scrub gate CLEAN, 20 files) from portfolio-demo f2afe53:
the downloadable interchange file and the field manifest no longer carry the rent tracker's
vendor-derived community unit counts (labelled "Internal pipeline only" with the reason), the
comps Built column and manifest years read 1984 instead of 1,984, and the Demand tab credits
"Home values: Zillow Home Value Index (ZHVI), Zillow Group" under the home-value table.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/downloads/underwriting-demo/sample-deal-summary.xlsx
+++ b/public/downloads/underwriting-demo/sample-deal-summary.xlsx
@@ -3502,7 +3502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I106"/>
+  <dimension ref="A1:I107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -4610,139 +4610,124 @@
         <v>-0.1242759499897198</v>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="4" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>Home values: Zillow Home Value Index (ZHVI), Zillow Group</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
         <is>
           <t>Labor market</t>
         </is>
       </c>
-      <c r="B57" s="4" t="n"/>
-      <c r="C57" s="4" t="n"/>
-      <c r="D57" s="4" t="n"/>
-      <c r="E57" s="4" t="n"/>
-      <c r="F57" s="4" t="n"/>
-      <c r="G57" s="4" t="n"/>
-      <c r="H57" s="4" t="n"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="6" t="inlineStr">
+      <c r="B58" s="4" t="n"/>
+      <c r="C58" s="4" t="n"/>
+      <c r="D58" s="4" t="n"/>
+      <c r="E58" s="4" t="n"/>
+      <c r="F58" s="4" t="n"/>
+      <c r="G58" s="4" t="n"/>
+      <c r="H58" s="4" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="inlineStr">
         <is>
           <t>Ring job counts are WORKPLACE counts — jobs located inside the ring, not residents who hold jobs. The unemployment row above is the opposite: residents. The two answer different questions and are not interchangeable.</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="14" t="inlineStr"/>
-      <c r="B59" s="14" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="14" t="inlineStr"/>
+      <c r="B60" s="14" t="inlineStr">
         <is>
           <t>1 mi</t>
         </is>
       </c>
-      <c r="C59" s="14" t="inlineStr">
+      <c r="C60" s="14" t="inlineStr">
         <is>
           <t>3 mi</t>
         </is>
       </c>
-      <c r="D59" s="14" t="inlineStr">
+      <c r="D60" s="14" t="inlineStr">
         <is>
           <t>5 mi</t>
         </is>
       </c>
-      <c r="E59" s="14" t="inlineStr">
+      <c r="E60" s="14" t="inlineStr">
         <is>
           <t>10 mi</t>
         </is>
       </c>
-      <c r="F59" s="14" t="inlineStr">
+      <c r="F60" s="14" t="inlineStr">
         <is>
           <t>Phoenix MSA</t>
         </is>
       </c>
-      <c r="G59" s="14" t="inlineStr">
+      <c r="G60" s="14" t="inlineStr">
         <is>
           <t>Arizona</t>
         </is>
       </c>
-      <c r="H59" s="14" t="inlineStr">
+      <c r="H60" s="14" t="inlineStr">
         <is>
           <t>U.S.</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="5" t="inlineStr">
+    <row r="61">
+      <c r="A61" s="5" t="inlineStr">
         <is>
           <t>Unemployment rate (residents, ACS)</t>
         </is>
       </c>
-      <c r="B60" s="11" t="n">
+      <c r="B61" s="11" t="n">
         <v>0.052</v>
       </c>
-      <c r="C60" s="11" t="n">
+      <c r="C61" s="11" t="n">
         <v>0.046</v>
       </c>
-      <c r="D60" s="11" t="n">
+      <c r="D61" s="11" t="n">
         <v>0.045</v>
       </c>
-      <c r="E60" s="11" t="n">
+      <c r="E61" s="11" t="n">
         <v>0.043</v>
       </c>
-      <c r="F60" s="11" t="n">
+      <c r="F61" s="11" t="n">
         <v>0.047</v>
       </c>
-      <c r="G60" s="11" t="n">
+      <c r="G61" s="11" t="n">
         <v>0.051</v>
       </c>
-      <c r="H60" s="11" t="n">
+      <c r="H61" s="11" t="n">
         <v>0.052</v>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="13" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="13" t="inlineStr">
         <is>
           <t>Jobs located inside the ring — LODES workplace counts</t>
         </is>
       </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    2019</t>
-        </is>
-      </c>
-      <c r="B62" s="7" t="n">
-        <v>4140</v>
-      </c>
-      <c r="C62" s="7" t="n">
-        <v>59139</v>
-      </c>
-      <c r="D62" s="7" t="n">
-        <v>150089</v>
-      </c>
-      <c r="E62" s="7" t="n">
-        <v>458614</v>
-      </c>
-      <c r="F62" s="12" t="n"/>
-      <c r="G62" s="12" t="n"/>
-      <c r="H62" s="12" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    2020</t>
+          <t xml:space="preserve">    2019</t>
         </is>
       </c>
       <c r="B63" s="7" t="n">
-        <v>4549</v>
+        <v>4140</v>
       </c>
       <c r="C63" s="7" t="n">
-        <v>58261</v>
+        <v>59139</v>
       </c>
       <c r="D63" s="7" t="n">
-        <v>150082</v>
+        <v>150089</v>
       </c>
       <c r="E63" s="7" t="n">
-        <v>455835</v>
+        <v>458614</v>
       </c>
       <c r="F63" s="12" t="n"/>
       <c r="G63" s="12" t="n"/>
@@ -4751,20 +4736,20 @@
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    2021</t>
+          <t xml:space="preserve">    2020</t>
         </is>
       </c>
       <c r="B64" s="7" t="n">
-        <v>4552</v>
+        <v>4549</v>
       </c>
       <c r="C64" s="7" t="n">
-        <v>59079</v>
+        <v>58261</v>
       </c>
       <c r="D64" s="7" t="n">
-        <v>152118</v>
+        <v>150082</v>
       </c>
       <c r="E64" s="7" t="n">
-        <v>466392</v>
+        <v>455835</v>
       </c>
       <c r="F64" s="12" t="n"/>
       <c r="G64" s="12" t="n"/>
@@ -4773,20 +4758,20 @@
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    2022</t>
+          <t xml:space="preserve">    2021</t>
         </is>
       </c>
       <c r="B65" s="7" t="n">
-        <v>4741</v>
+        <v>4552</v>
       </c>
       <c r="C65" s="7" t="n">
-        <v>63403</v>
+        <v>59079</v>
       </c>
       <c r="D65" s="7" t="n">
-        <v>162056</v>
+        <v>152118</v>
       </c>
       <c r="E65" s="7" t="n">
-        <v>501214</v>
+        <v>466392</v>
       </c>
       <c r="F65" s="12" t="n"/>
       <c r="G65" s="12" t="n"/>
@@ -4795,20 +4780,20 @@
     <row r="66">
       <c r="A66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    2023  (latest)</t>
+          <t xml:space="preserve">    2022</t>
         </is>
       </c>
       <c r="B66" s="7" t="n">
-        <v>5239</v>
+        <v>4741</v>
       </c>
       <c r="C66" s="7" t="n">
-        <v>65083</v>
+        <v>63403</v>
       </c>
       <c r="D66" s="7" t="n">
-        <v>165142</v>
+        <v>162056</v>
       </c>
       <c r="E66" s="7" t="n">
-        <v>516916</v>
+        <v>501214</v>
       </c>
       <c r="F66" s="12" t="n"/>
       <c r="G66" s="12" t="n"/>
@@ -4817,947 +4802,969 @@
     <row r="67">
       <c r="A67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Job growth 2019 to 2023</t>
-        </is>
-      </c>
-      <c r="B67" s="11" t="n">
-        <v>0.2654589371980676</v>
-      </c>
-      <c r="C67" s="11" t="n">
-        <v>0.1005089703917887</v>
-      </c>
-      <c r="D67" s="11" t="n">
-        <v>0.1002938256634396</v>
-      </c>
-      <c r="E67" s="11" t="n">
-        <v>0.1271265159807595</v>
+          <t xml:space="preserve">    2023  (latest)</t>
+        </is>
+      </c>
+      <c r="B67" s="7" t="n">
+        <v>5239</v>
+      </c>
+      <c r="C67" s="7" t="n">
+        <v>65083</v>
+      </c>
+      <c r="D67" s="7" t="n">
+        <v>165142</v>
+      </c>
+      <c r="E67" s="7" t="n">
+        <v>516916</v>
       </c>
       <c r="F67" s="12" t="n"/>
       <c r="G67" s="12" t="n"/>
       <c r="H67" s="12" t="n"/>
-      <c r="I67" s="2" t="inlineStr">
-        <is>
-          <t>Already a fraction in the engine's output, unlike the rates above.</t>
-        </is>
-      </c>
     </row>
     <row r="68">
       <c r="A68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Job CAGR (4-yr)</t>
+          <t xml:space="preserve">    Job growth 2019 to 2023</t>
         </is>
       </c>
       <c r="B68" s="11" t="n">
-        <v>0.06062537773196808</v>
+        <v>0.2654589371980676</v>
       </c>
       <c r="C68" s="11" t="n">
-        <v>0.02423213297708893</v>
+        <v>0.1005089703917887</v>
       </c>
       <c r="D68" s="11" t="n">
-        <v>0.02418207107245318</v>
+        <v>0.1002938256634396</v>
       </c>
       <c r="E68" s="11" t="n">
-        <v>0.03036990821614882</v>
+        <v>0.1271265159807595</v>
       </c>
       <c r="F68" s="12" t="n"/>
       <c r="G68" s="12" t="n"/>
       <c r="H68" s="12" t="n"/>
-    </row>
-    <row r="70">
-      <c r="A70" s="13" t="inlineStr">
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>Already a fraction in the engine's output, unlike the rates above.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Job CAGR (4-yr)</t>
+        </is>
+      </c>
+      <c r="B69" s="11" t="n">
+        <v>0.06062537773196808</v>
+      </c>
+      <c r="C69" s="11" t="n">
+        <v>0.02423213297708893</v>
+      </c>
+      <c r="D69" s="11" t="n">
+        <v>0.02418207107245318</v>
+      </c>
+      <c r="E69" s="11" t="n">
+        <v>0.03036990821614882</v>
+      </c>
+      <c r="F69" s="12" t="n"/>
+      <c r="G69" s="12" t="n"/>
+      <c r="H69" s="12" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="13" t="inlineStr">
         <is>
           <t>Metro nonfarm employment and unemployment — Maricopa County, Arizona</t>
         </is>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" s="14" t="inlineStr">
+    <row r="72">
+      <c r="A72" s="14" t="inlineStr">
         <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="B71" s="14" t="inlineStr">
+      <c r="B72" s="14" t="inlineStr">
         <is>
           <t>Nonfarm jobs (000s)</t>
         </is>
       </c>
-      <c r="C71" s="14" t="inlineStr">
+      <c r="C72" s="14" t="inlineStr">
         <is>
           <t>Job growth</t>
         </is>
       </c>
-      <c r="D71" s="14" t="inlineStr">
+      <c r="D72" s="14" t="inlineStr">
         <is>
           <t>Unemployment</t>
         </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="12" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B72" s="10" t="n">
-        <v>2469.37</v>
-      </c>
-      <c r="C72" s="11" t="n">
-        <v>0.002793919975309533</v>
-      </c>
-      <c r="D72" s="11" t="n">
-        <v>0.0431</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="12" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B73" s="10" t="n">
-        <v>2462.49</v>
+        <v>2469.37</v>
       </c>
       <c r="C73" s="11" t="n">
-        <v>0.002626178726730766</v>
+        <v>0.002793919975309533</v>
       </c>
       <c r="D73" s="11" t="n">
-        <v>0.0381</v>
+        <v>0.0431</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="12" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B74" s="10" t="n">
-        <v>2456.04</v>
+        <v>2462.49</v>
       </c>
       <c r="C74" s="11" t="n">
-        <v>0.02243406947942472</v>
+        <v>0.002626178726730766</v>
       </c>
       <c r="D74" s="11" t="n">
-        <v>0.0328</v>
+        <v>0.0381</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="12" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B75" s="10" t="n">
-        <v>2402.15</v>
+        <v>2456.04</v>
       </c>
       <c r="C75" s="11" t="n">
-        <v>0.03166081866321946</v>
+        <v>0.02243406947942472</v>
       </c>
       <c r="D75" s="11" t="n">
-        <v>0.0326</v>
+        <v>0.0328</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="12" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="B76" s="10" t="n">
-        <v>2328.43</v>
+        <v>2402.15</v>
       </c>
       <c r="C76" s="11" t="n">
-        <v>0.05041323059710923</v>
+        <v>0.03166081866321946</v>
       </c>
       <c r="D76" s="11" t="n">
-        <v>0.0332</v>
+        <v>0.0326</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="12" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="B77" s="10" t="n">
-        <v>2216.68</v>
+        <v>2328.43</v>
       </c>
       <c r="C77" s="11" t="n">
-        <v>0.04558897751446889</v>
+        <v>0.05041323059710923</v>
       </c>
       <c r="D77" s="11" t="n">
-        <v>0.0462</v>
+        <v>0.0332</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="12" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="B78" s="10" t="n">
-        <v>2120.03</v>
+        <v>2216.68</v>
       </c>
       <c r="C78" s="11" t="n">
-        <v>-0.02628980328576602</v>
+        <v>0.04558897751446889</v>
       </c>
       <c r="D78" s="11" t="n">
-        <v>0.0728</v>
+        <v>0.0462</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="12" t="n">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="B79" s="10" t="n">
-        <v>2177.27</v>
+        <v>2120.03</v>
       </c>
       <c r="C79" s="11" t="n">
-        <v>0.03380213477170857</v>
+        <v>-0.02628980328576602</v>
       </c>
       <c r="D79" s="11" t="n">
-        <v>0.0413</v>
+        <v>0.0728</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="12" t="n">
-        <v>2018</v>
+        <v>2019</v>
       </c>
       <c r="B80" s="10" t="n">
-        <v>2106.08</v>
+        <v>2177.27</v>
       </c>
       <c r="C80" s="11" t="n">
-        <v>0.03344079531681654</v>
+        <v>0.03380213477170857</v>
       </c>
       <c r="D80" s="11" t="n">
-        <v>0.0415</v>
+        <v>0.0413</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="12" t="n">
-        <v>2017</v>
+        <v>2018</v>
       </c>
       <c r="B81" s="10" t="n">
-        <v>2037.93</v>
+        <v>2106.08</v>
       </c>
       <c r="C81" s="11" t="n">
-        <v>0.03009517840264042</v>
+        <v>0.03344079531681654</v>
       </c>
       <c r="D81" s="11" t="n">
-        <v>0.0428</v>
+        <v>0.0415</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="12" t="n">
+        <v>2017</v>
+      </c>
+      <c r="B82" s="10" t="n">
+        <v>2037.93</v>
+      </c>
+      <c r="C82" s="11" t="n">
+        <v>0.03009517840264042</v>
+      </c>
+      <c r="D82" s="11" t="n">
+        <v>0.0428</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="12" t="n">
         <v>2016</v>
       </c>
-      <c r="B82" s="10" t="n">
+      <c r="B83" s="10" t="n">
         <v>1978.39</v>
       </c>
-      <c r="C82" s="12" t="n"/>
-      <c r="D82" s="11" t="n">
+      <c r="C83" s="12" t="n"/>
+      <c r="D83" s="11" t="n">
         <v>0.0471</v>
       </c>
     </row>
-    <row r="84">
-      <c r="A84" s="4" t="inlineStr">
+    <row r="85">
+      <c r="A85" s="4" t="inlineStr">
         <is>
           <t>Jobs by industry (2023)</t>
         </is>
       </c>
-      <c r="B84" s="4" t="n"/>
-      <c r="C84" s="4" t="n"/>
-      <c r="D84" s="4" t="n"/>
-      <c r="E84" s="4" t="n"/>
-      <c r="F84" s="4" t="n"/>
-      <c r="G84" s="4" t="n"/>
-      <c r="H84" s="4" t="n"/>
-    </row>
-    <row r="85">
-      <c r="A85" s="6" t="inlineStr">
+      <c r="B85" s="4" t="n"/>
+      <c r="C85" s="4" t="n"/>
+      <c r="D85" s="4" t="n"/>
+      <c r="E85" s="4" t="n"/>
+      <c r="F85" s="4" t="n"/>
+      <c r="G85" s="4" t="n"/>
+      <c r="H85" s="4" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="6" t="inlineStr">
         <is>
           <t>Share of jobs by sector, sorted by the metro's own concentration. Ring, MSA and state shares come from LODES workplace counts; the U.S. column is QCEW — a different survey, so read it as a benchmark rather than the same measurement. The location quotient on each row is the metro share over the national share.</t>
         </is>
       </c>
     </row>
-    <row r="86">
-      <c r="A86" s="14" t="inlineStr"/>
-      <c r="B86" s="14" t="inlineStr">
+    <row r="87">
+      <c r="A87" s="14" t="inlineStr"/>
+      <c r="B87" s="14" t="inlineStr">
         <is>
           <t>1 mi</t>
         </is>
       </c>
-      <c r="C86" s="14" t="inlineStr">
+      <c r="C87" s="14" t="inlineStr">
         <is>
           <t>3 mi</t>
         </is>
       </c>
-      <c r="D86" s="14" t="inlineStr">
+      <c r="D87" s="14" t="inlineStr">
         <is>
           <t>5 mi</t>
         </is>
       </c>
-      <c r="E86" s="14" t="inlineStr">
+      <c r="E87" s="14" t="inlineStr">
         <is>
           <t>10 mi</t>
         </is>
       </c>
-      <c r="F86" s="14" t="inlineStr">
+      <c r="F87" s="14" t="inlineStr">
         <is>
           <t>Phoenix MSA</t>
         </is>
       </c>
-      <c r="G86" s="14" t="inlineStr">
+      <c r="G87" s="14" t="inlineStr">
         <is>
           <t>Arizona</t>
         </is>
       </c>
-      <c r="H86" s="14" t="inlineStr">
+      <c r="H87" s="14" t="inlineStr">
         <is>
           <t>U.S.</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" s="5" t="inlineStr">
-        <is>
-          <t>Health Care/Social Asst</t>
-        </is>
-      </c>
-      <c r="B87" s="11" t="n">
-        <v>0.1675892345867532</v>
-      </c>
-      <c r="C87" s="11" t="n">
-        <v>0.1324022003011585</v>
-      </c>
-      <c r="D87" s="11" t="n">
-        <v>0.128294871717239</v>
-      </c>
-      <c r="E87" s="11" t="n">
-        <v>0.1575223875399726</v>
-      </c>
-      <c r="F87" s="11" t="n">
-        <v>0.1439230188830762</v>
-      </c>
-      <c r="G87" s="11" t="n">
-        <v>0.1480747084992491</v>
-      </c>
-      <c r="H87" s="11" t="n">
-        <v>0.1524112221376376</v>
-      </c>
-      <c r="I87" s="2" t="inlineStr">
-        <is>
-          <t>Location quotient vs U.S.: 0.94x — less concentrated here.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="5" t="inlineStr">
         <is>
-          <t>Retail Trade</t>
+          <t>Health Care/Social Asst</t>
         </is>
       </c>
       <c r="B88" s="11" t="n">
-        <v>0.1402939492269517</v>
+        <v>0.1675892345867532</v>
       </c>
       <c r="C88" s="11" t="n">
-        <v>0.1312959036292677</v>
+        <v>0.1324022003011585</v>
       </c>
       <c r="D88" s="11" t="n">
-        <v>0.1295604415567115</v>
+        <v>0.128294871717239</v>
       </c>
       <c r="E88" s="11" t="n">
-        <v>0.1260357078602561</v>
+        <v>0.1575223875399726</v>
       </c>
       <c r="F88" s="11" t="n">
-        <v>0.1090536545703669</v>
+        <v>0.1439230188830762</v>
       </c>
       <c r="G88" s="11" t="n">
-        <v>0.1100206596769526</v>
+        <v>0.1480747084992491</v>
       </c>
       <c r="H88" s="11" t="n">
-        <v>0.1019921721752688</v>
+        <v>0.1524112221376376</v>
       </c>
       <c r="I88" s="2" t="inlineStr">
         <is>
-          <t>Location quotient vs U.S.: 1.07x — more concentrated here.</t>
+          <t>Location quotient vs U.S.: 0.94x — less concentrated here.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="5" t="inlineStr">
         <is>
-          <t>Accommodation/Food Svcs</t>
+          <t>Retail Trade</t>
         </is>
       </c>
       <c r="B89" s="11" t="n">
-        <v>0.1093720175606032</v>
+        <v>0.1402939492269517</v>
       </c>
       <c r="C89" s="11" t="n">
-        <v>0.09160751052518361</v>
+        <v>0.1312959036292677</v>
       </c>
       <c r="D89" s="11" t="n">
-        <v>0.09612275421907074</v>
+        <v>0.1295604415567115</v>
       </c>
       <c r="E89" s="11" t="n">
-        <v>0.0974934080326242</v>
+        <v>0.1260357078602561</v>
       </c>
       <c r="F89" s="11" t="n">
-        <v>0.09153364975214603</v>
+        <v>0.1090536545703669</v>
       </c>
       <c r="G89" s="11" t="n">
-        <v>0.09799831322286184</v>
+        <v>0.1100206596769526</v>
       </c>
       <c r="H89" s="11" t="n">
-        <v>0.09210003364899073</v>
+        <v>0.1019921721752688</v>
       </c>
       <c r="I89" s="2" t="inlineStr">
         <is>
-          <t>Location quotient vs U.S.: 0.99x — less concentrated here.</t>
+          <t>Location quotient vs U.S.: 1.07x — more concentrated here.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="5" t="inlineStr">
         <is>
-          <t>Admin/Support/Waste</t>
+          <t>Accommodation/Food Svcs</t>
         </is>
       </c>
       <c r="B90" s="11" t="n">
-        <v>0.09200229051345676</v>
+        <v>0.1093720175606032</v>
       </c>
       <c r="C90" s="11" t="n">
-        <v>0.1102148059371255</v>
+        <v>0.09160751052518361</v>
       </c>
       <c r="D90" s="11" t="n">
-        <v>0.09007950685163767</v>
+        <v>0.09612275421907074</v>
       </c>
       <c r="E90" s="11" t="n">
-        <v>0.07061675278623067</v>
+        <v>0.0974934080326242</v>
       </c>
       <c r="F90" s="11" t="n">
-        <v>0.08654896600644772</v>
+        <v>0.09153364975214603</v>
       </c>
       <c r="G90" s="11" t="n">
-        <v>0.08053357937738248</v>
+        <v>0.09799831322286184</v>
       </c>
       <c r="H90" s="11" t="n">
-        <v>0.06170694540515537</v>
+        <v>0.09210003364899073</v>
       </c>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t>Location quotient vs U.S.: 1.40x — more concentrated here.</t>
+          <t>Location quotient vs U.S.: 0.99x — less concentrated here.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="5" t="inlineStr">
         <is>
-          <t>Construction</t>
+          <t>Admin/Support/Waste</t>
         </is>
       </c>
       <c r="B91" s="11" t="n">
-        <v>0.03397594960870395</v>
+        <v>0.09200229051345676</v>
       </c>
       <c r="C91" s="11" t="n">
-        <v>0.1437571064195937</v>
+        <v>0.1102148059371255</v>
       </c>
       <c r="D91" s="11" t="n">
-        <v>0.1065198040486124</v>
+        <v>0.09007950685163767</v>
       </c>
       <c r="E91" s="11" t="n">
-        <v>0.07423822393150158</v>
+        <v>0.07061675278623067</v>
       </c>
       <c r="F91" s="11" t="n">
-        <v>0.07168567465967132</v>
+        <v>0.08654896600644772</v>
       </c>
       <c r="G91" s="11" t="n">
-        <v>0.0692629280579044</v>
+        <v>0.08053357937738248</v>
       </c>
       <c r="H91" s="11" t="n">
-        <v>0.0531750429082045</v>
+        <v>0.06170694540515537</v>
       </c>
       <c r="I91" s="2" t="inlineStr">
         <is>
-          <t>Location quotient vs U.S.: 1.35x — more concentrated here.</t>
+          <t>Location quotient vs U.S.: 1.40x — more concentrated here.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="5" t="inlineStr">
         <is>
-          <t>Educational Services</t>
+          <t>Construction</t>
         </is>
       </c>
       <c r="B92" s="11" t="n">
-        <v>0.05630845581217789</v>
+        <v>0.03397594960870395</v>
       </c>
       <c r="C92" s="11" t="n">
-        <v>0.09185335423004824</v>
+        <v>0.1437571064195937</v>
       </c>
       <c r="D92" s="11" t="n">
-        <v>0.1103528457155314</v>
+        <v>0.1065198040486124</v>
       </c>
       <c r="E92" s="11" t="n">
-        <v>0.09778359001541834</v>
+        <v>0.07423822393150158</v>
       </c>
       <c r="F92" s="11" t="n">
-        <v>0.0692937123890178</v>
+        <v>0.07168567465967132</v>
       </c>
       <c r="G92" s="11" t="n">
-        <v>0.07805244418719343</v>
+        <v>0.0692629280579044</v>
       </c>
       <c r="H92" s="11" t="n">
-        <v>0.08463384936674581</v>
+        <v>0.0531750429082045</v>
       </c>
       <c r="I92" s="2" t="inlineStr">
         <is>
-          <t>Location quotient vs U.S.: 0.82x — less concentrated here.</t>
+          <t>Location quotient vs U.S.: 1.35x — more concentrated here.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="5" t="inlineStr">
         <is>
-          <t>Finance/Insurance</t>
+          <t>Educational Services</t>
         </is>
       </c>
       <c r="B93" s="11" t="n">
-        <v>0.01355220461920214</v>
+        <v>0.05630845581217789</v>
       </c>
       <c r="C93" s="11" t="n">
-        <v>0.02564457146369196</v>
+        <v>0.09185335423004824</v>
       </c>
       <c r="D93" s="11" t="n">
-        <v>0.02846623835100489</v>
+        <v>0.1103528457155314</v>
       </c>
       <c r="E93" s="11" t="n">
-        <v>0.06430626193373404</v>
+        <v>0.09778359001541834</v>
       </c>
       <c r="F93" s="11" t="n">
-        <v>0.06699836548547758</v>
+        <v>0.0692937123890178</v>
       </c>
       <c r="G93" s="11" t="n">
-        <v>0.05584002806837911</v>
+        <v>0.07805244418719343</v>
       </c>
       <c r="H93" s="11" t="n">
-        <v>0.04139724841428747</v>
+        <v>0.08463384936674581</v>
       </c>
       <c r="I93" s="2" t="inlineStr">
         <is>
-          <t>Location quotient vs U.S.: 1.62x — more concentrated here.</t>
+          <t>Location quotient vs U.S.: 0.82x — less concentrated here.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="5" t="inlineStr">
         <is>
-          <t>Manufacturing</t>
+          <t>Finance/Insurance</t>
         </is>
       </c>
       <c r="B94" s="11" t="n">
-        <v>0.005344531399121969</v>
+        <v>0.01355220461920214</v>
       </c>
       <c r="C94" s="11" t="n">
-        <v>0.03838234842199072</v>
+        <v>0.02564457146369196</v>
       </c>
       <c r="D94" s="11" t="n">
-        <v>0.04546362849167086</v>
+        <v>0.02846623835100489</v>
       </c>
       <c r="E94" s="11" t="n">
-        <v>0.06499302595968018</v>
+        <v>0.06430626193373404</v>
       </c>
       <c r="F94" s="11" t="n">
-        <v>0.06180957654864814</v>
+        <v>0.06699836548547758</v>
       </c>
       <c r="G94" s="11" t="n">
-        <v>0.06178450068945185</v>
+        <v>0.05584002806837911</v>
       </c>
       <c r="H94" s="11" t="n">
-        <v>0.08451882031580928</v>
+        <v>0.04139724841428747</v>
       </c>
       <c r="I94" s="2" t="inlineStr">
         <is>
-          <t>Location quotient vs U.S.: 0.73x — less concentrated here.</t>
+          <t>Location quotient vs U.S.: 1.62x — more concentrated here.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="5" t="inlineStr">
         <is>
-          <t>Professional/Scientific/Tech</t>
+          <t>Manufacturing</t>
         </is>
       </c>
       <c r="B95" s="11" t="n">
-        <v>0.03531208245848445</v>
+        <v>0.005344531399121969</v>
       </c>
       <c r="C95" s="11" t="n">
-        <v>0.06550198211487047</v>
+        <v>0.03838234842199072</v>
       </c>
       <c r="D95" s="11" t="n">
-        <v>0.05942728423245309</v>
+        <v>0.04546362849167086</v>
       </c>
       <c r="E95" s="11" t="n">
-        <v>0.06130384568509065</v>
+        <v>0.06499302595968018</v>
       </c>
       <c r="F95" s="11" t="n">
-        <v>0.06005544300027939</v>
+        <v>0.06180957654864814</v>
       </c>
       <c r="G95" s="11" t="n">
-        <v>0.05671111569578283</v>
+        <v>0.06178450068945185</v>
       </c>
       <c r="H95" s="11" t="n">
-        <v>0.07101058481218332</v>
+        <v>0.08451882031580928</v>
       </c>
       <c r="I95" s="2" t="inlineStr">
         <is>
-          <t>Location quotient vs U.S.: 0.85x — less concentrated here.</t>
+          <t>Location quotient vs U.S.: 0.73x — less concentrated here.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="5" t="inlineStr">
         <is>
-          <t>Transportation/Warehousing</t>
+          <t>Professional/Scientific/Tech</t>
         </is>
       </c>
       <c r="B96" s="11" t="n">
-        <v>0.01068906279824394</v>
+        <v>0.03531208245848445</v>
       </c>
       <c r="C96" s="11" t="n">
-        <v>0.006038536000737531</v>
+        <v>0.06550198211487047</v>
       </c>
       <c r="D96" s="11" t="n">
-        <v>0.01906832260525726</v>
+        <v>0.05942728423245309</v>
       </c>
       <c r="E96" s="11" t="n">
-        <v>0.02301916942178338</v>
+        <v>0.06130384568509065</v>
       </c>
       <c r="F96" s="11" t="n">
-        <v>0.0473268911935302</v>
+        <v>0.06005544300027939</v>
       </c>
       <c r="G96" s="11" t="n">
-        <v>0.04326179016785311</v>
+        <v>0.05671111569578283</v>
       </c>
       <c r="H96" s="11" t="n">
-        <v>0.04840196213219566</v>
+        <v>0.07101058481218332</v>
       </c>
       <c r="I96" s="2" t="inlineStr">
         <is>
-          <t>Location quotient vs U.S.: 0.98x — less concentrated here.</t>
+          <t>Location quotient vs U.S.: 0.85x — less concentrated here.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="5" t="inlineStr">
         <is>
-          <t>Wholesale Trade</t>
+          <t>Transportation/Warehousing</t>
         </is>
       </c>
       <c r="B97" s="11" t="n">
-        <v>0.007825920977285742</v>
+        <v>0.01068906279824394</v>
       </c>
       <c r="C97" s="11" t="n">
-        <v>0.03606219845733075</v>
+        <v>0.006038536000737531</v>
       </c>
       <c r="D97" s="11" t="n">
-        <v>0.03811847913626373</v>
+        <v>0.01906832260525726</v>
       </c>
       <c r="E97" s="11" t="n">
-        <v>0.03247329842121656</v>
+        <v>0.02301916942178338</v>
       </c>
       <c r="F97" s="11" t="n">
-        <v>0.04109248140049621</v>
+        <v>0.0473268911935302</v>
       </c>
       <c r="G97" s="11" t="n">
-        <v>0.03708044284108286</v>
+        <v>0.04326179016785311</v>
       </c>
       <c r="H97" s="11" t="n">
-        <v>0.03992451539947575</v>
+        <v>0.04840196213219566</v>
       </c>
       <c r="I97" s="2" t="inlineStr">
         <is>
-          <t>Location quotient vs U.S.: 1.03x — more concentrated here.</t>
+          <t>Location quotient vs U.S.: 0.98x — less concentrated here.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="5" t="inlineStr">
         <is>
-          <t>Public Administration</t>
+          <t>Wholesale Trade</t>
         </is>
       </c>
       <c r="B98" s="11" t="n">
-        <v>0</v>
+        <v>0.007825920977285742</v>
       </c>
       <c r="C98" s="11" t="n">
-        <v>0.001859193018038782</v>
+        <v>0.03606219845733075</v>
       </c>
       <c r="D98" s="11" t="n">
-        <v>0.02761848821930085</v>
+        <v>0.03811847913626373</v>
       </c>
       <c r="E98" s="11" t="n">
-        <v>0.02183329238543132</v>
+        <v>0.03247329842121656</v>
       </c>
       <c r="F98" s="11" t="n">
-        <v>0.03285591679200175</v>
+        <v>0.04109248140049621</v>
       </c>
       <c r="G98" s="11" t="n">
-        <v>0.04120792091186574</v>
+        <v>0.03708044284108286</v>
       </c>
       <c r="H98" s="11" t="n">
-        <v>0.04966983338636385</v>
+        <v>0.03992451539947575</v>
       </c>
       <c r="I98" s="2" t="inlineStr">
         <is>
-          <t>Location quotient vs U.S.: 0.66x — less concentrated here.</t>
+          <t>Location quotient vs U.S.: 1.03x — more concentrated here.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="5" t="inlineStr">
         <is>
-          <t>Other Services</t>
+          <t>Public Administration</t>
         </is>
       </c>
       <c r="B99" s="11" t="n">
-        <v>0.01546096583317427</v>
+        <v>0</v>
       </c>
       <c r="C99" s="11" t="n">
-        <v>0.02945514888909376</v>
+        <v>0.001859193018038782</v>
       </c>
       <c r="D99" s="11" t="n">
-        <v>0.03031917792458657</v>
+        <v>0.02761848821930085</v>
       </c>
       <c r="E99" s="11" t="n">
-        <v>0.02663677147395037</v>
+        <v>0.02183329238543132</v>
       </c>
       <c r="F99" s="11" t="n">
-        <v>0.02745633069056147</v>
+        <v>0.03285591679200175</v>
       </c>
       <c r="G99" s="11" t="n">
-        <v>0.02813810432102126</v>
+        <v>0.04120792091186574</v>
       </c>
       <c r="H99" s="11" t="n">
-        <v>0.03015265325357227</v>
+        <v>0.04966983338636385</v>
       </c>
       <c r="I99" s="2" t="inlineStr">
         <is>
-          <t>Location quotient vs U.S.: 0.91x — less concentrated here.</t>
+          <t>Location quotient vs U.S.: 0.66x — less concentrated here.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="5" t="inlineStr">
         <is>
-          <t>Arts/Entertainment/Rec</t>
+          <t>Other Services</t>
         </is>
       </c>
       <c r="B100" s="11" t="n">
-        <v>0.2744798625691926</v>
+        <v>0.01546096583317427</v>
       </c>
       <c r="C100" s="11" t="n">
-        <v>0.03211333394794259</v>
+        <v>0.02945514888909376</v>
       </c>
       <c r="D100" s="11" t="n">
-        <v>0.0287326741066833</v>
+        <v>0.03031917792458657</v>
       </c>
       <c r="E100" s="11" t="n">
-        <v>0.02107301559051066</v>
+        <v>0.02663677147395037</v>
       </c>
       <c r="F100" s="11" t="n">
-        <v>0.02090656164729619</v>
+        <v>0.02745633069056147</v>
       </c>
       <c r="G100" s="11" t="n">
-        <v>0.02117990984115704</v>
+        <v>0.02813810432102126</v>
       </c>
       <c r="H100" s="11" t="n">
-        <v>0.01844252444674844</v>
+        <v>0.03015265325357227</v>
       </c>
       <c r="I100" s="2" t="inlineStr">
         <is>
-          <t>Location quotient vs U.S.: 1.13x — more concentrated here.</t>
+          <t>Location quotient vs U.S.: 0.91x — less concentrated here.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="5" t="inlineStr">
         <is>
-          <t>Real Estate/Rental</t>
+          <t>Arts/Entertainment/Rec</t>
         </is>
       </c>
       <c r="B101" s="11" t="n">
-        <v>0.03340332124451231</v>
+        <v>0.2744798625691926</v>
       </c>
       <c r="C101" s="11" t="n">
-        <v>0.03411081404996773</v>
+        <v>0.03211333394794259</v>
       </c>
       <c r="D101" s="11" t="n">
-        <v>0.02407610374039469</v>
+        <v>0.0287326741066833</v>
       </c>
       <c r="E101" s="11" t="n">
-        <v>0.02037464428525276</v>
+        <v>0.02107301559051066</v>
       </c>
       <c r="F101" s="11" t="n">
-        <v>0.02084382439592392</v>
+        <v>0.02090656164729619</v>
       </c>
       <c r="G101" s="11" t="n">
-        <v>0.01961125167587262</v>
+        <v>0.02117990984115704</v>
       </c>
       <c r="H101" s="11" t="n">
-        <v>0.01586685774361</v>
+        <v>0.01844252444674844</v>
       </c>
       <c r="I101" s="2" t="inlineStr">
         <is>
-          <t>Location quotient vs U.S.: 1.31x — more concentrated here.</t>
+          <t>Location quotient vs U.S.: 1.13x — more concentrated here.</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="5" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Real Estate/Rental</t>
         </is>
       </c>
       <c r="B102" s="11" t="n">
-        <v>0.002672265699560985</v>
+        <v>0.03340332124451231</v>
       </c>
       <c r="C102" s="11" t="n">
-        <v>0.01090931440336806</v>
+        <v>0.03411081404996773</v>
       </c>
       <c r="D102" s="11" t="n">
-        <v>0.01293424486657018</v>
+        <v>0.02407610374039469</v>
       </c>
       <c r="E102" s="11" t="n">
-        <v>0.01705883149519169</v>
+        <v>0.02037464428525276</v>
       </c>
       <c r="F102" s="11" t="n">
-        <v>0.01906250470529385</v>
+        <v>0.02084382439592392</v>
       </c>
       <c r="G102" s="11" t="n">
-        <v>0.01736157873170788</v>
+        <v>0.01961125167587262</v>
       </c>
       <c r="H102" s="11" t="n">
-        <v>0.02037764401856688</v>
+        <v>0.01586685774361</v>
       </c>
       <c r="I102" s="2" t="inlineStr">
         <is>
-          <t>Location quotient vs U.S.: 0.94x — less concentrated here.</t>
+          <t>Location quotient vs U.S.: 1.31x — more concentrated here.</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="5" t="inlineStr">
         <is>
-          <t>Mgmt of Companies</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="B103" s="11" t="n">
-        <v>0.0005726283641916397</v>
+        <v>0.002672265699560985</v>
       </c>
       <c r="C103" s="11" t="n">
-        <v>0.01676346762545712</v>
+        <v>0.01090931440336806</v>
       </c>
       <c r="D103" s="11" t="n">
-        <v>0.01896538151783606</v>
+        <v>0.01293424486657018</v>
       </c>
       <c r="E103" s="11" t="n">
-        <v>0.01917522542303697</v>
+        <v>0.01705883149519169</v>
       </c>
       <c r="F103" s="11" t="n">
-        <v>0.01809509628913341</v>
+        <v>0.01906250470529385</v>
       </c>
       <c r="G103" s="11" t="n">
-        <v>0.01520137056214125</v>
+        <v>0.01736157873170788</v>
       </c>
       <c r="H103" s="11" t="n">
-        <v>0.0166872404072684</v>
+        <v>0.02037764401856688</v>
       </c>
       <c r="I103" s="2" t="inlineStr">
         <is>
-          <t>Location quotient vs U.S.: 1.08x — more concentrated here.</t>
+          <t>Location quotient vs U.S.: 0.94x — less concentrated here.</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="5" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Mgmt of Companies</t>
         </is>
       </c>
       <c r="B104" s="11" t="n">
-        <v>0.001145256728383279</v>
+        <v>0.0005726283641916397</v>
       </c>
       <c r="C104" s="11" t="n">
-        <v>0.0007221658830398574</v>
+        <v>0.01676346762545712</v>
       </c>
       <c r="D104" s="11" t="n">
-        <v>0.003772488086082971</v>
+        <v>0.01896538151783606</v>
       </c>
       <c r="E104" s="11" t="n">
-        <v>0.002512975970997278</v>
+        <v>0.01917522542303697</v>
       </c>
       <c r="F104" s="11" t="n">
-        <v>0.006769767671410718</v>
+        <v>0.01809509628913341</v>
       </c>
       <c r="G104" s="11" t="n">
-        <v>0.006825111647899759</v>
+        <v>0.01520137056214125</v>
       </c>
       <c r="H104" s="11" t="n">
-        <v>0.0054838649167028</v>
+        <v>0.0166872404072684</v>
       </c>
       <c r="I104" s="2" t="inlineStr">
         <is>
-          <t>Location quotient vs U.S.: 1.23x — more concentrated here.</t>
+          <t>Location quotient vs U.S.: 1.08x — more concentrated here.</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="5" t="inlineStr">
         <is>
-          <t>Agriculture/Forestry/Fishing</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="B105" s="11" t="n">
-        <v>0</v>
+        <v>0.001145256728383279</v>
       </c>
       <c r="C105" s="11" t="n">
-        <v>0.0006299744937156203</v>
+        <v>0.0007221658830398574</v>
       </c>
       <c r="D105" s="11" t="n">
-        <v>0.001725777053826078</v>
+        <v>0.003772488086082971</v>
       </c>
       <c r="E105" s="11" t="n">
-        <v>0.001151055198416767</v>
+        <v>0.002512975970997278</v>
       </c>
       <c r="F105" s="11" t="n">
-        <v>0.003239751660864168</v>
+        <v>0.006769767671410718</v>
       </c>
       <c r="G105" s="11" t="n">
-        <v>0.007704795534784445</v>
+        <v>0.006825111647899759</v>
       </c>
       <c r="H105" s="11" t="n">
-        <v>0.008224135502638645</v>
+        <v>0.0054838649167028</v>
       </c>
       <c r="I105" s="2" t="inlineStr">
         <is>
-          <t>Location quotient vs U.S.: 0.39x — less concentrated here.</t>
+          <t>Location quotient vs U.S.: 1.23x — more concentrated here.</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="5" t="inlineStr">
         <is>
-          <t>Mining/Oil &amp; Gas</t>
+          <t>Agriculture/Forestry/Fishing</t>
         </is>
       </c>
       <c r="B106" s="11" t="n">
         <v>0</v>
       </c>
       <c r="C106" s="11" t="n">
+        <v>0.0006299744937156203</v>
+      </c>
+      <c r="D106" s="11" t="n">
+        <v>0.001725777053826078</v>
+      </c>
+      <c r="E106" s="11" t="n">
+        <v>0.001151055198416767</v>
+      </c>
+      <c r="F106" s="11" t="n">
+        <v>0.003239751660864168</v>
+      </c>
+      <c r="G106" s="11" t="n">
+        <v>0.007704795534784445</v>
+      </c>
+      <c r="H106" s="11" t="n">
+        <v>0.008224135502638645</v>
+      </c>
+      <c r="I106" s="2" t="inlineStr">
+        <is>
+          <t>Location quotient vs U.S.: 0.39x — less concentrated here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="5" t="inlineStr">
+        <is>
+          <t>Mining/Oil &amp; Gas</t>
+        </is>
+      </c>
+      <c r="B107" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C107" s="11" t="n">
         <v>0.0006760701883777388</v>
       </c>
-      <c r="D106" s="11" t="n">
+      <c r="D107" s="11" t="n">
         <v>0.0003814875592668172</v>
       </c>
-      <c r="E106" s="11" t="n">
+      <c r="E107" s="11" t="n">
         <v>0.0003985165897039564</v>
       </c>
-      <c r="F106" s="11" t="n">
+      <c r="F107" s="11" t="n">
         <v>0.00144881225835702</v>
       </c>
-      <c r="G106" s="11" t="n">
+      <c r="G107" s="11" t="n">
         <v>0.004149446289456433</v>
       </c>
-      <c r="H106" s="11" t="n">
+      <c r="H107" s="11" t="n">
         <v>0.003822849608574414</v>
       </c>
-      <c r="I106" s="2" t="inlineStr">
+      <c r="I107" s="2" t="inlineStr">
         <is>
           <t>Location quotient vs U.S.: 0.38x — less concentrated here.</t>
         </is>
@@ -8776,7 +8783,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H60"/>
+  <dimension ref="A1:H61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -8826,7 +8833,7 @@
         </is>
       </c>
       <c r="B5" s="23" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6">
@@ -8984,22 +8991,22 @@
     <row r="12">
       <c r="A12" s="24" t="inlineStr">
         <is>
-          <t>comps.rows</t>
+          <t>comps.nearby[].units</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>19 entries</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Operator's own weekly rent scrape, via the market-report service</t>
+          <t>Internal pipeline only</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>POST /report (format json)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -9010,94 +9017,94 @@
       <c r="F12" s="12" t="n"/>
       <c r="G12" s="22" t="inlineStr">
         <is>
-          <t>Own weekly scrape; asking and net effective stated separately.</t>
+          <t>Unit counts come from a licensed data export; the internal pipeline carries them.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="24" t="inlineStr">
         <is>
-          <t>comps.rows.tier</t>
+          <t>comps.rows</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>19 entries</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Tracked-community registry, via the market-report service</t>
+          <t>Operator's own weekly rent scrape, via the market-report service</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>comp_tiers.assign</t>
+          <t>POST /report (format json)</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>derived</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>comps.rows.distance_mi, comps.tiering.subject_product, comps.tiering.subject_year_built, comps.tiering.year_band, comps.tiering.top_n, comps.tiering.additional_n</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F13" s="12" t="n"/>
       <c r="G13" s="22" t="inlineStr">
         <is>
-          <t>Closest same-product communities first, within the vintage band where the registry carries a year built; an unknown year keeps the community and says so.</t>
+          <t>Own weekly scrape; asking and net effective stated separately.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="24" t="inlineStr">
         <is>
-          <t>demand.rings</t>
+          <t>comps.rows.tier</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>5 entries</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Public demographic data (the operator's ring engine), via the market-report service</t>
+          <t>Tracked-community registry, via the market-report service</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>POST /report (format json)</t>
+          <t>comp_tiers.assign</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>read</t>
-        </is>
-      </c>
-      <c r="F14" s="12" t="n"/>
+          <t>derived</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>comps.rows.distance_mi, comps.tiering.subject_product, comps.tiering.subject_year_built, comps.tiering.year_band, comps.tiering.top_n, comps.tiering.additional_n</t>
+        </is>
+      </c>
       <c r="G14" s="22" t="inlineStr">
         <is>
-          <t>Ring demographics.</t>
+          <t>Closest same-product communities first, within the vintage band where the registry carries a year built; an unknown year keeps the community and says so.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="24" t="inlineStr">
         <is>
-          <t>demand.zip_home</t>
+          <t>demand.rings</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>5 entries</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Zillow ZHVI home values (vendored static table, undated), via the market-report service</t>
+          <t>Public demographic data (the operator's ring engine), via the market-report service</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
@@ -9113,29 +9120,29 @@
       <c r="F15" s="12" t="n"/>
       <c r="G15" s="22" t="inlineStr">
         <is>
-          <t>ZIP and metro home values from the vendored Zillow ZHVI table; static, undated.</t>
+          <t>Ring demographics.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="24" t="inlineStr">
         <is>
-          <t>om_comps.rent</t>
+          <t>demand.zip_home</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>0 entries</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Sample Property Offering Memorandum.pdf</t>
+          <t>Zillow ZHVI home values (vendored static table, undated), via the market-report service</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>p.20</t>
+          <t>POST /report (format json)</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -9146,29 +9153,29 @@
       <c r="F16" s="12" t="n"/>
       <c r="G16" s="22" t="inlineStr">
         <is>
-          <t>4 rent comparable(s) the memorandum states; every figure verified inside its own quote.</t>
+          <t>ZIP and metro home values from the vendored Zillow ZHVI table; static, undated.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="24" t="inlineStr">
         <is>
-          <t>pricing.price_per_unit</t>
+          <t>om_comps.rent</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>215,000</t>
+          <t>0 entries</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Illustrative price</t>
+          <t>Sample Property Offering Memorandum.pdf</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>p.20</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -9179,24 +9186,24 @@
       <c r="F17" s="12" t="n"/>
       <c r="G17" s="22" t="inlineStr">
         <is>
-          <t>Per-unit price chosen for the sample, inside the sale-price band; every cap rate and pricing ladder is computed from it.</t>
+          <t>4 rent comparable(s) the memorandum states; every figure verified inside its own quote.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="24" t="inlineStr">
         <is>
-          <t>pricing.unit_count</t>
+          <t>pricing.price_per_unit</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>334</t>
+          <t>215,000</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Sample Property RR 8.4.26.xlsx</t>
+          <t>Illustrative price</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
@@ -9206,34 +9213,30 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>derived</t>
-        </is>
-      </c>
-      <c r="F18" s="5" t="inlineStr">
-        <is>
-          <t>summary.unit_count</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F18" s="12" t="n"/>
       <c r="G18" s="22" t="inlineStr">
         <is>
-          <t>The same count the summary carries, counted from the rows of the uploaded rent roll.</t>
+          <t>Per-unit price chosen for the sample, inside the sale-price band; every cap rate and pricing ladder is computed from it.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="24" t="inlineStr">
         <is>
-          <t>summary.address_provenance</t>
+          <t>pricing.unit_count</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Illustrative address — not the asset's real location. The market tabs were pulled for t…</t>
+          <t>334</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Illustrative address</t>
+          <t>Sample Property RR 8.4.26.xlsx</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
@@ -9243,30 +9246,34 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>read</t>
-        </is>
-      </c>
-      <c r="F19" s="12" t="n"/>
+          <t>derived</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>summary.unit_count</t>
+        </is>
+      </c>
       <c r="G19" s="22" t="inlineStr">
         <is>
-          <t>Illustrative address — not the asset's real location. The market tabs were pulled for this address on 2026-09-14.</t>
+          <t>The same count the summary carries, counted from the rows of the uploaded rent roll.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="24" t="inlineStr">
         <is>
-          <t>summary.assessed_value_basis</t>
+          <t>summary.address_provenance</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>Illustrative address — not the asset's real location. The market tabs were pulled for t…</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>Internal pipeline only</t>
+          <t>Illustrative address</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
@@ -9282,29 +9289,29 @@
       <c r="F20" s="12" t="n"/>
       <c r="G20" s="22" t="inlineStr">
         <is>
-          <t>See parcel: read off the county assessor's portal by the internal pipeline only.</t>
+          <t>Illustrative address — not the asset's real location. The market tabs were pulled for this address on 2026-09-14.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="24" t="inlineStr">
         <is>
-          <t>summary.assessment_ratio</t>
+          <t>summary.assessed_value_basis</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>0.1</t>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Vendored county rate table</t>
+          <t>Internal pipeline only</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>property_tax_table.STATE_RULES['AZ']</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
@@ -9315,29 +9322,29 @@
       <c r="F21" s="12" t="n"/>
       <c r="G21" s="22" t="inlineStr">
         <is>
-          <t>10% — legal class 4.2, residential rental. A.R.S. sec. 42-15003 (class four assessed at 10%); A.R.S. sec. 42-12004 (class four includes residential rental property).</t>
+          <t>See parcel: read off the county assessor's portal by the internal pipeline only.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="24" t="inlineStr">
         <is>
-          <t>summary.city</t>
+          <t>summary.assessment_ratio</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Mesa</t>
+          <t>0.1</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Illustrative address</t>
+          <t>Vendored county rate table</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>property_tax_table.STATE_RULES['AZ']</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
@@ -9348,24 +9355,24 @@
       <c r="F22" s="12" t="n"/>
       <c r="G22" s="22" t="inlineStr">
         <is>
-          <t>Illustrative address — not the asset's real location. The market tabs were pulled for this address on 2026-09-14.</t>
+          <t>10% — legal class 4.2, residential rental. A.R.S. sec. 42-15003 (class four assessed at 10%); A.R.S. sec. 42-12004 (class four includes residential rental property).</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="24" t="inlineStr">
         <is>
-          <t>summary.construction_status</t>
+          <t>summary.city</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>Mesa</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Not stated in the uploaded documents</t>
+          <t>Illustrative address</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
@@ -9381,24 +9388,24 @@
       <c r="F23" s="12" t="n"/>
       <c r="G23" s="22" t="inlineStr">
         <is>
-          <t>No uploaded document stated this, so the value reads MISSING. Nothing was assumed to fill it.</t>
+          <t>Illustrative address — not the asset's real location. The market tabs were pulled for this address on 2026-09-14.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="24" t="inlineStr">
         <is>
-          <t>summary.county</t>
+          <t>summary.construction_status</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Maricopa</t>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Illustrative address</t>
+          <t>Not stated in the uploaded documents</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
@@ -9414,24 +9421,24 @@
       <c r="F24" s="12" t="n"/>
       <c r="G24" s="22" t="inlineStr">
         <is>
-          <t>Illustrative address — not the asset's real location. The market tabs were pulled for this address on 2026-09-14.</t>
+          <t>No uploaded document stated this, so the value reads MISSING. Nothing was assumed to fill it.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="24" t="inlineStr">
         <is>
-          <t>summary.deal_name</t>
+          <t>summary.county</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Sample Mesa Apt</t>
+          <t>Maricopa</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Illustrative name</t>
+          <t>Illustrative address</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
@@ -9447,24 +9454,24 @@
       <c r="F25" s="12" t="n"/>
       <c r="G25" s="22" t="inlineStr">
         <is>
-          <t>An illustrative name for the public sample. The real asset's name is withheld; the memorandum's own name for it does not appear anywhere in this set.</t>
+          <t>Illustrative address — not the asset's real location. The market tabs were pulled for this address on 2026-09-14.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="24" t="inlineStr">
         <is>
-          <t>summary.deal_status</t>
+          <t>summary.deal_name</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>Sample Mesa Apt</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Not stated in the uploaded documents</t>
+          <t>Illustrative name</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
@@ -9480,14 +9487,14 @@
       <c r="F26" s="12" t="n"/>
       <c r="G26" s="22" t="inlineStr">
         <is>
-          <t>No uploaded document stated this, so the value reads MISSING. Nothing was assumed to fill it.</t>
+          <t>An illustrative name for the public sample. The real asset's name is withheld; the memorandum's own name for it does not appear anywhere in this set.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="24" t="inlineStr">
         <is>
-          <t>summary.delivery_date</t>
+          <t>summary.deal_status</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
@@ -9520,7 +9527,7 @@
     <row r="28">
       <c r="A28" s="24" t="inlineStr">
         <is>
-          <t>summary.fair_market_value</t>
+          <t>summary.delivery_date</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
@@ -9530,7 +9537,7 @@
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Internal pipeline only</t>
+          <t>Not stated in the uploaded documents</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
@@ -9546,24 +9553,24 @@
       <c r="F28" s="12" t="n"/>
       <c r="G28" s="22" t="inlineStr">
         <is>
-          <t>The internal pipeline pulls a market value by web lookup; the demo does not reach the web.</t>
+          <t>No uploaded document stated this, so the value reads MISSING. Nothing was assumed to fill it.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="24" t="inlineStr">
         <is>
-          <t>summary.in_place_rent_avg</t>
+          <t>summary.fair_market_value</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>1,456.99</t>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Sample Property RR 8.4.26.xlsx</t>
+          <t>Internal pipeline only</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
@@ -9573,34 +9580,30 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>derived</t>
-        </is>
-      </c>
-      <c r="F29" s="5" t="inlineStr">
-        <is>
-          <t>rent_roll.units</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F29" s="12" t="n"/>
       <c r="G29" s="22" t="inlineStr">
         <is>
-          <t>Unit-weighted across the uploaded roll.</t>
+          <t>The internal pipeline pulls a market value by web lookup; the demo does not reach the web.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="24" t="inlineStr">
         <is>
-          <t>summary.listing_brokerage</t>
+          <t>summary.in_place_rent_avg</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Desert Ridge Capital Advisors</t>
+          <t>1,456.99</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>Illustrative name</t>
+          <t>Sample Property RR 8.4.26.xlsx</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
@@ -9610,30 +9613,34 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>read</t>
-        </is>
-      </c>
-      <c r="F30" s="12" t="n"/>
+          <t>derived</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>rent_roll.units</t>
+        </is>
+      </c>
       <c r="G30" s="22" t="inlineStr">
         <is>
-          <t>An illustrative name. The real party is withheld from the public sample.</t>
+          <t>Unit-weighted across the uploaded roll.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="24" t="inlineStr">
         <is>
-          <t>summary.market_rent_for_model</t>
+          <t>summary.listing_brokerage</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>1,344.6</t>
+          <t>Desert Ridge Capital Advisors</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Sample Property RR 8.4.26.xlsx</t>
+          <t>Illustrative name</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
@@ -9643,34 +9650,30 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>derived</t>
-        </is>
-      </c>
-      <c r="F31" s="5" t="inlineStr">
-        <is>
-          <t>rent_roll.units</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F31" s="12" t="n"/>
       <c r="G31" s="22" t="inlineStr">
         <is>
-          <t>Unit-weighted across the uploaded roll.</t>
+          <t>An illustrative name. The real party is withheld from the public sample.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="24" t="inlineStr">
         <is>
-          <t>summary.msa</t>
+          <t>summary.market_rent_for_model</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Phoenix MSA</t>
+          <t>1,344.6</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>Illustrative address</t>
+          <t>Sample Property RR 8.4.26.xlsx</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
@@ -9680,30 +9683,34 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>read</t>
-        </is>
-      </c>
-      <c r="F32" s="12" t="n"/>
+          <t>derived</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>rent_roll.units</t>
+        </is>
+      </c>
       <c r="G32" s="22" t="inlineStr">
         <is>
-          <t>Illustrative address — not the asset's real location. The market tabs were pulled for this address on 2026-09-14.</t>
+          <t>Unit-weighted across the uploaded roll.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="24" t="inlineStr">
         <is>
-          <t>summary.pricing_guidance</t>
+          <t>summary.msa</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>$215,000 per unit (illustrative)</t>
+          <t>Phoenix MSA</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Illustrative price</t>
+          <t>Illustrative address</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
@@ -9719,29 +9726,29 @@
       <c r="F33" s="12" t="n"/>
       <c r="G33" s="22" t="inlineStr">
         <is>
-          <t>Every price and cap rate below is illustrative. The per-unit price is a round number chosen for the sample inside the band a real per-unit sale price occupies; it is not a quote, an offer, or a broker's guidance.</t>
+          <t>Illustrative address — not the asset's real location. The market tabs were pulled for this address on 2026-09-14.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="24" t="inlineStr">
         <is>
-          <t>summary.product_detail</t>
+          <t>summary.pricing_guidance</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>Diversified mix of one-, two-, and three-bedroom residences averaging 856 square feet o…</t>
+          <t>$215,000 per unit (illustrative)</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>Sample Property Offering Memorandum.pdf</t>
+          <t>Illustrative price</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>p.3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -9751,6 +9758,39 @@
       </c>
       <c r="F34" s="12" t="n"/>
       <c r="G34" s="22" t="inlineStr">
+        <is>
+          <t>Every price and cap rate below is illustrative. The per-unit price is a round number chosen for the sample inside the band a real per-unit sale price occupies; it is not a quote, an offer, or a broker's guidance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="24" t="inlineStr">
+        <is>
+          <t>summary.product_detail</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>Diversified mix of one-, two-, and three-bedroom residences averaging 856 square feet o…</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>Sample Property Offering Memorandum.pdf</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>p.3</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F35" s="12" t="n"/>
+      <c r="G35" s="22" t="inlineStr">
         <is>
           <t>the property offers a diversified mix of 
 one-, two-, and three-bedroom residences averaging 856 square 
@@ -9758,58 +9798,25 @@
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="24" t="inlineStr">
-        <is>
-          <t>summary.product_type</t>
-        </is>
-      </c>
-      <c r="B35" s="5" t="inlineStr">
-        <is>
-          <t>Garden-style multifamily</t>
-        </is>
-      </c>
-      <c r="C35" s="5" t="inlineStr">
-        <is>
-          <t>Sample Property Offering Memorandum.pdf</t>
-        </is>
-      </c>
-      <c r="D35" s="5" t="inlineStr">
-        <is>
-          <t>p.3</t>
-        </is>
-      </c>
-      <c r="E35" s="5" t="inlineStr">
-        <is>
-          <t>read</t>
-        </is>
-      </c>
-      <c r="F35" s="12" t="n"/>
-      <c r="G35" s="22" t="inlineStr">
-        <is>
-          <t>Stated in the memorandum; withheld from the public sample because it identifies the real asset.</t>
-        </is>
-      </c>
-    </row>
     <row r="36">
       <c r="A36" s="24" t="inlineStr">
         <is>
-          <t>summary.school_elementary_name</t>
+          <t>summary.product_type</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>Porter Elementary School</t>
+          <t>Garden-style multifamily</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>Internal underwriting agent — attendance-zone school lookup</t>
+          <t>Sample Property Offering Memorandum.pdf</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>2151 E Southern Ave, Mesa, AZ 85204 on 2026-09-14</t>
+          <t>p.3</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -9820,19 +9827,19 @@
       <c r="F36" s="12" t="n"/>
       <c r="G36" s="22" t="inlineStr">
         <is>
-          <t>Looked up for the illustrative address by the internal underwriting agent; the public demo does not run this on an uploaded deal.</t>
+          <t>Stated in the memorandum; withheld from the public sample because it identifies the real asset.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="24" t="inlineStr">
         <is>
-          <t>summary.school_high_name</t>
+          <t>summary.school_elementary_name</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>Mesa High School</t>
+          <t>Porter Elementary School</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
@@ -9860,12 +9867,12 @@
     <row r="38">
       <c r="A38" s="24" t="inlineStr">
         <is>
-          <t>summary.school_middle_name</t>
+          <t>summary.school_high_name</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>Taylor Junior High School</t>
+          <t>Mesa High School</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
@@ -9893,22 +9900,22 @@
     <row r="39">
       <c r="A39" s="24" t="inlineStr">
         <is>
-          <t>summary.seller_entity</t>
+          <t>summary.school_middle_name</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>Sonoran Residential Holdings LLC</t>
+          <t>Taylor Junior High School</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Illustrative name</t>
+          <t>Internal underwriting agent — attendance-zone school lookup</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2151 E Southern Ave, Mesa, AZ 85204 on 2026-09-14</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
@@ -9919,24 +9926,24 @@
       <c r="F39" s="12" t="n"/>
       <c r="G39" s="22" t="inlineStr">
         <is>
-          <t>An illustrative name. The real party is withheld from the public sample.</t>
+          <t>Looked up for the illustrative address by the internal underwriting agent; the public demo does not run this on an uploaded deal.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="24" t="inlineStr">
         <is>
-          <t>summary.state</t>
+          <t>summary.seller_entity</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>Sonoran Residential Holdings LLC</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>Illustrative address</t>
+          <t>Illustrative name</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
@@ -9952,19 +9959,19 @@
       <c r="F40" s="12" t="n"/>
       <c r="G40" s="22" t="inlineStr">
         <is>
-          <t>Illustrative address — not the asset's real location. The market tabs were pulled for this address on 2026-09-14.</t>
+          <t>An illustrative name. The real party is withheld from the public sample.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="24" t="inlineStr">
         <is>
-          <t>summary.street_address</t>
+          <t>summary.state</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>2151 E Southern Ave</t>
+          <t>AZ</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
@@ -9992,22 +9999,22 @@
     <row r="42">
       <c r="A42" s="24" t="inlineStr">
         <is>
-          <t>summary.structure</t>
+          <t>summary.street_address</t>
         </is>
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>1 &amp; 2 stories</t>
+          <t>2151 E Southern Ave</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>Sample Property Offering Memorandum.pdf</t>
+          <t>Illustrative address</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>p.10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
@@ -10018,29 +10025,29 @@
       <c r="F42" s="12" t="n"/>
       <c r="G42" s="22" t="inlineStr">
         <is>
-          <t>Number of Stories 1 &amp; 2</t>
+          <t>Illustrative address — not the asset's real location. The market tabs were pulled for this address on 2026-09-14.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="24" t="inlineStr">
         <is>
-          <t>summary.tax_area_code</t>
+          <t>summary.structure</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>1 &amp; 2 stories</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>Internal pipeline only</t>
+          <t>Sample Property Offering Memorandum.pdf</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>p.10</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
@@ -10051,29 +10058,29 @@
       <c r="F43" s="12" t="n"/>
       <c r="G43" s="22" t="inlineStr">
         <is>
-          <t>See parcel: read off the county assessor's portal by the internal pipeline only.</t>
+          <t>Number of Stories 1 &amp; 2</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="24" t="inlineStr">
         <is>
-          <t>summary.tax_basis_label</t>
+          <t>summary.tax_area_code</t>
         </is>
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>Limited property value (LPV), per the county assessor</t>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>Vendored county rate table</t>
+          <t>Internal pipeline only</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>property_tax_table.STATE_RULES['AZ']</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
@@ -10084,19 +10091,19 @@
       <c r="F44" s="12" t="n"/>
       <c r="G44" s="22" t="inlineStr">
         <is>
-          <t>What the assessed basis is in this state.</t>
+          <t>See parcel: read off the county assessor's portal by the internal pipeline only.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="24" t="inlineStr">
         <is>
-          <t>summary.tax_basis_note</t>
+          <t>summary.tax_basis_label</t>
         </is>
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>Arizona taxes the limited property value, not the price. Under Proposition 117 (Ariz. C…</t>
+          <t>Limited property value (LPV), per the county assessor</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
@@ -10117,29 +10124,29 @@
       <c r="F45" s="12" t="n"/>
       <c r="G45" s="22" t="inlineStr">
         <is>
-          <t>How the basis behaves on a sale, with the authority.</t>
+          <t>What the assessed basis is in this state.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="24" t="inlineStr">
         <is>
-          <t>summary.tax_billed_amount</t>
+          <t>summary.tax_basis_note</t>
         </is>
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>249,122</t>
+          <t>Arizona taxes the limited property value, not the price. Under Proposition 117 (Ariz. C…</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>Sample Property Offering Memorandum.pdf</t>
+          <t>Vendored county rate table</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>p.10</t>
+          <t>property_tax_table.STATE_RULES['AZ']</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
@@ -10150,19 +10157,19 @@
       <c r="F46" s="12" t="n"/>
       <c r="G46" s="22" t="inlineStr">
         <is>
-          <t>2025 Property Tax $249,122</t>
+          <t>How the basis behaves on a sale, with the authority.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="24" t="inlineStr">
         <is>
-          <t>summary.tax_billed_year</t>
+          <t>summary.tax_billed_amount</t>
         </is>
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>2,025</t>
+          <t>249,122</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
@@ -10190,22 +10197,22 @@
     <row r="48">
       <c r="A48" s="24" t="inlineStr">
         <is>
-          <t>summary.tax_divisor</t>
+          <t>summary.tax_billed_year</t>
         </is>
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>2,025</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>Vendored county rate table</t>
+          <t>Sample Property Offering Memorandum.pdf</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>property_tax_table.STATE_RULES['AZ']</t>
+          <t>p.10</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
@@ -10216,29 +10223,29 @@
       <c r="F48" s="12" t="n"/>
       <c r="G48" s="22" t="inlineStr">
         <is>
-          <t>The rate's unit in Arizona: per $100 of assessed value.</t>
+          <t>2025 Property Tax $249,122</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="24" t="inlineStr">
         <is>
-          <t>summary.tax_exemption</t>
+          <t>summary.tax_divisor</t>
         </is>
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>100</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>Internal pipeline only</t>
+          <t>Vendored county rate table</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>property_tax_table.STATE_RULES['AZ']</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
@@ -10249,29 +10256,29 @@
       <c r="F49" s="12" t="n"/>
       <c r="G49" s="22" t="inlineStr">
         <is>
-          <t>See parcel: read off the county assessor's portal by the internal pipeline only.</t>
+          <t>The rate's unit in Arizona: per $100 of assessed value.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="24" t="inlineStr">
         <is>
-          <t>summary.tax_parcel_id</t>
+          <t>summary.tax_exemption</t>
         </is>
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>301-04-002K</t>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>Sample Property Offering Memorandum.pdf</t>
+          <t>Internal pipeline only</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>p.10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
@@ -10282,56 +10289,52 @@
       <c r="F50" s="12" t="n"/>
       <c r="G50" s="22" t="inlineStr">
         <is>
-          <t>Tax Parcel Number 301-04-002K</t>
+          <t>See parcel: read off the county assessor's portal by the internal pipeline only.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="24" t="inlineStr">
         <is>
-          <t>summary.tax_per_unit_flag</t>
+          <t>summary.tax_parcel_id</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>In band (the statement's line per unit): $717 per unit a year is inside the AZ band of …</t>
+          <t>301-04-002K</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>Vendored county rate table</t>
+          <t>Sample Property Offering Memorandum.pdf</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>property_tax_table.band_check</t>
+          <t>p.10</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
         <is>
-          <t>derived</t>
-        </is>
-      </c>
-      <c r="F51" s="5" t="inlineStr">
-        <is>
-          <t>summary.tax_statement_amount, summary.unit_count, summary.state</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F51" s="12" t="n"/>
       <c r="G51" s="22" t="inlineStr">
         <is>
-          <t>A sanity check against the state's typical per-unit range. It flags; it never changes a figure.</t>
+          <t>Tax Parcel Number 301-04-002K</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="24" t="inlineStr">
         <is>
-          <t>summary.tax_rate_as_billed</t>
+          <t>summary.tax_per_unit_flag</t>
         </is>
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>10.26</t>
+          <t>In band (the statement's line per unit): $717 per unit a year is inside the AZ band of …</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
@@ -10341,30 +10344,34 @@
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>property_tax_table.COUNTY_RATES[('AZ', 'maricopa')]</t>
+          <t>property_tax_table.band_check</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t>read</t>
-        </is>
-      </c>
-      <c r="F52" s="12" t="n"/>
+          <t>derived</t>
+        </is>
+      </c>
+      <c r="F52" s="5" t="inlineStr">
+        <is>
+          <t>summary.tax_statement_amount, summary.unit_count, summary.state</t>
+        </is>
+      </c>
       <c r="G52" s="22" t="inlineStr">
         <is>
-          <t>Tax area code 971300 — City of Phoenix / Deer Valley Unified School District #97, tax year 2025. Maricopa County, '2025 Tax Rates, Maricopa County, Arizona' (the treasurer's rate table by tax area code), row 971300: primary 6.7007, approx residential primary 5.1401, secondary 3.5566. Verified 2026-09-04.</t>
+          <t>A sanity check against the state's typical per-unit range. It flags; it never changes a figure.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="24" t="inlineStr">
         <is>
-          <t>summary.tax_rate_evidence</t>
+          <t>summary.tax_rate_as_billed</t>
         </is>
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>Vendored county rate table: 10.2573 per $100 of assessed value, tax year 2025 — Tax are…</t>
+          <t>10.26</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
@@ -10374,34 +10381,30 @@
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>property_tax_table.evidence_text</t>
+          <t>property_tax_table.COUNTY_RATES[('AZ', 'maricopa')]</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t>derived</t>
-        </is>
-      </c>
-      <c r="F53" s="5" t="inlineStr">
-        <is>
-          <t>summary.state, summary.county, summary.tax_parcel_id, summary.tax_billed_amount, summary.tax_billed_year</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F53" s="12" t="n"/>
       <c r="G53" s="22" t="inlineStr">
         <is>
-          <t>The citation, tax year and jurisdiction stack behind the rate, or the honest note that none is on file. Also records what the uploaded document stated for the field(s) it cites.</t>
+          <t>Tax area code 971300 — City of Phoenix / Deer Valley Unified School District #97, tax year 2025. Maricopa County, '2025 Tax Rates, Maricopa County, Arizona' (the treasurer's rate table by tax area code), row 971300: primary 6.7007, approx residential primary 5.1401, secondary 3.5566. Verified 2026-09-04.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="24" t="inlineStr">
         <is>
-          <t>summary.tax_rate_year</t>
+          <t>summary.tax_rate_evidence</t>
         </is>
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>2,025</t>
+          <t>Vendored county rate table: 10.2573 per $100 of assessed value, tax year 2025 — Tax are…</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
@@ -10411,147 +10414,151 @@
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>property_tax_table.COUNTY_RATES[('AZ', 'maricopa')]</t>
+          <t>property_tax_table.evidence_text</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t>read</t>
-        </is>
-      </c>
-      <c r="F54" s="12" t="n"/>
+          <t>derived</t>
+        </is>
+      </c>
+      <c r="F54" s="5" t="inlineStr">
+        <is>
+          <t>summary.state, summary.county, summary.tax_parcel_id, summary.tax_billed_amount, summary.tax_billed_year</t>
+        </is>
+      </c>
       <c r="G54" s="22" t="inlineStr">
         <is>
-          <t>The tax year of the rate on file. A bill from another year is displayed, not tied out.</t>
+          <t>The citation, tax year and jurisdiction stack behind the rate, or the honest note that none is on file. Also records what the uploaded document stated for the field(s) it cites.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="24" t="inlineStr">
         <is>
-          <t>summary.tax_statement_amount</t>
+          <t>summary.tax_rate_year</t>
         </is>
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>239,566.79</t>
+          <t>2,025</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>Sample Property T-12 June 26.xlsx</t>
+          <t>Vendored county rate table</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>Property Taxes lines</t>
+          <t>property_tax_table.COUNTY_RATES[('AZ', 'maricopa')]</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t>computed</t>
-        </is>
-      </c>
-      <c r="F55" s="5" t="inlineStr">
-        <is>
-          <t>t12.rows</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F55" s="12" t="n"/>
       <c r="G55" s="22" t="inlineStr">
         <is>
-          <t>The statement's lines categorised as Property Taxes, summed over its twelve months. As billed in the statement, not the county's bill.</t>
+          <t>The tax year of the rate on file. A bill from another year is displayed, not tied out.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="24" t="inlineStr">
         <is>
-          <t>summary.unit_count</t>
+          <t>summary.tax_statement_amount</t>
         </is>
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>334</t>
+          <t>239,566.79</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>Sample Property RR 8.4.26.xlsx</t>
+          <t>Sample Property T-12 June 26.xlsx</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Property Taxes lines</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t>derived</t>
+          <t>computed</t>
         </is>
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>rent_roll.units</t>
+          <t>t12.rows</t>
         </is>
       </c>
       <c r="G56" s="22" t="inlineStr">
         <is>
-          <t>Counted from the rows of the uploaded rent roll.</t>
+          <t>The statement's lines categorised as Property Taxes, summed over its twelve months. As billed in the statement, not the county's bill.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="24" t="inlineStr">
         <is>
-          <t>summary.year_built</t>
+          <t>summary.unit_count</t>
         </is>
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>1,981</t>
+          <t>334</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>Sample Property Offering Memorandum.pdf</t>
+          <t>Sample Property RR 8.4.26.xlsx</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>p.10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t>read</t>
-        </is>
-      </c>
-      <c r="F57" s="12" t="n"/>
+          <t>derived</t>
+        </is>
+      </c>
+      <c r="F57" s="5" t="inlineStr">
+        <is>
+          <t>rent_roll.units</t>
+        </is>
+      </c>
       <c r="G57" s="22" t="inlineStr">
         <is>
-          <t>Y ear Built 1981</t>
+          <t>Counted from the rows of the uploaded rent roll.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="24" t="inlineStr">
         <is>
-          <t>summary.zip</t>
+          <t>summary.year_built</t>
         </is>
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>85204</t>
+          <t>1,981</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>Illustrative address</t>
+          <t>Sample Property Offering Memorandum.pdf</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>p.10</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr">
@@ -10562,75 +10569,108 @@
       <c r="F58" s="12" t="n"/>
       <c r="G58" s="22" t="inlineStr">
         <is>
-          <t>Illustrative address — not the asset's real location. The market tabs were pulled for this address on 2026-09-14.</t>
+          <t>Y ear Built 1981</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="24" t="inlineStr">
         <is>
-          <t>supply.projects</t>
+          <t>summary.zip</t>
         </is>
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>32 entries</t>
+          <t>85204</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>Public permit and entitlement records (the operator's supply pipeline), via the market-report service</t>
+          <t>Illustrative address</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>POST /report (format json)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t>derived</t>
-        </is>
-      </c>
-      <c r="F59" s="5" t="inlineStr">
-        <is>
-          <t>supply.rings</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F59" s="12" t="n"/>
       <c r="G59" s="22" t="inlineStr">
         <is>
-          <t>The developments the counts are made of, within 3 mi: one row per development, reconciled across the pipeline's lifecycle layers and shown at the furthest stage any layer carries.</t>
+          <t>Illustrative address — not the asset's real location. The market tabs were pulled for this address on 2026-09-14.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="24" t="inlineStr">
         <is>
+          <t>supply.projects</t>
+        </is>
+      </c>
+      <c r="B60" s="5" t="inlineStr">
+        <is>
+          <t>32 entries</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>Public permit and entitlement records (the operator's supply pipeline), via the market-report service</t>
+        </is>
+      </c>
+      <c r="D60" s="5" t="inlineStr">
+        <is>
+          <t>POST /report (format json)</t>
+        </is>
+      </c>
+      <c r="E60" s="5" t="inlineStr">
+        <is>
+          <t>derived</t>
+        </is>
+      </c>
+      <c r="F60" s="5" t="inlineStr">
+        <is>
           <t>supply.rings</t>
         </is>
       </c>
-      <c r="B60" s="5" t="inlineStr">
+      <c r="G60" s="22" t="inlineStr">
+        <is>
+          <t>The developments the counts are made of, within 3 mi: one row per development, reconciled across the pipeline's lifecycle layers and shown at the furthest stage any layer carries.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="24" t="inlineStr">
+        <is>
+          <t>supply.rings</t>
+        </is>
+      </c>
+      <c r="B61" s="5" t="inlineStr">
         <is>
           <t>8 entries</t>
         </is>
       </c>
-      <c r="C60" s="5" t="inlineStr">
+      <c r="C61" s="5" t="inlineStr">
         <is>
           <t>Public permit and entitlement records (the operator's supply pipeline), via the market-report service</t>
         </is>
       </c>
-      <c r="D60" s="5" t="inlineStr">
+      <c r="D61" s="5" t="inlineStr">
         <is>
           <t>POST /report (format json)</t>
         </is>
       </c>
-      <c r="E60" s="5" t="inlineStr">
+      <c r="E61" s="5" t="inlineStr">
         <is>
           <t>read</t>
         </is>
       </c>
-      <c r="F60" s="12" t="n"/>
-      <c r="G60" s="22" t="inlineStr">
+      <c r="F61" s="12" t="n"/>
+      <c r="G61" s="22" t="inlineStr">
         <is>
           <t>Projects and units by cumulative ring and tracked stage, counted from the service's project rows.</t>
         </is>

</xml_diff>